<commit_message>
fix(case_d4): correct gate 3 boundaries and counts
</commit_message>
<xml_diff>
--- a/analysis/CASE_D4/CASE_D4_participant_workbook.xlsx
+++ b/analysis/CASE_D4/CASE_D4_participant_workbook.xlsx
@@ -541,14 +541,14 @@
         </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>7857</v>
+        <v>7856</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Q1;Q5</t>
+          <t>Q1;Q3;Q4;Q5</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -700,7 +700,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Q2;Q5</t>
+          <t>Q1;Q5</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -781,7 +781,7 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>dignity_autonomy;family_caregiver_ecology;age_dignity_language;balance_multidimensional;mental_health_elderly</t>
+          <t>dignity_autonomy;family_caregiver_ecology;age_dignity_language;balance_multidimensional;practical_suggestion</t>
         </is>
       </c>
     </row>
@@ -852,7 +852,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Q2;Q3;Q5;Q7</t>
+          <t>Q1;Q3;Q5;Q7</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -928,7 +928,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Q1;Q2;Q3;Q4;Q5;Q7</t>
+          <t>Q1;Q2;Q3;Q4;Q5;Q6;Q7</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -1004,7 +1004,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Q1;Q2;Q3;Q4;Q5;Q6;Q7</t>
+          <t>Q1;Q2;Q3;Q4;Q5;Q6</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -1042,7 +1042,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Q1;Q2;Q3;Q4;Q6</t>
+          <t>Q1;Q2;Q3;Q4;Q5</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -1080,7 +1080,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Q1;Q2;Q3;Q4</t>
+          <t>Q1;Q2;Q4;Q6</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -1232,7 +1232,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Q4;Q5</t>
+          <t>Q4;Q5;Q7</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -1270,7 +1270,7 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Q6;Q7</t>
+          <t>Q5;Q7</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -1453,19 +1453,19 @@
         </is>
       </c>
       <c r="E27" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>2601</v>
+        <v>2600</v>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Q1;Q2;Q4;Q5</t>
+          <t>Q1;Q2;Q3;Q4;Q5;Q7</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>technology_integration;balance_multidimensional;institutional_example;person_centered_care;cultural_barrier</t>
+          <t>balance_multidimensional;institutional_example;person_centered_care;cultural_barrier;dignity_autonomy</t>
         </is>
       </c>
     </row>
@@ -1498,12 +1498,12 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Q1;Q2;Q3</t>
+          <t>Q1;Q2;Q3;Q4</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>balance_multidimensional;technology_integration;dependence_resistance;dignity_autonomy;mental_health_elderly</t>
+          <t>balance_multidimensional;dependence_resistance;dignity_autonomy;mental_health_elderly;spiritual_moral_anchor</t>
         </is>
       </c>
     </row>
@@ -1529,19 +1529,19 @@
         </is>
       </c>
       <c r="E29" s="2" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>2568</v>
+        <v>2566</v>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Q1;Q2;Q3;Q5</t>
+          <t>Q1;Q2;Q3;Q4;Q5;Q6;Q7</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>technology_integration;awareness_education;balance_multidimensional;dependence_resistance;family_caregiver_ecology</t>
+          <t>awareness_education;balance_multidimensional;dependence_resistance;family_caregiver_ecology;home_care_services</t>
         </is>
       </c>
     </row>
@@ -1567,19 +1567,19 @@
         </is>
       </c>
       <c r="E30" s="2" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>2344</v>
+        <v>2339</v>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Q1;Q2;Q3;Q7</t>
+          <t>Q1;Q2;Q3;Q5;Q6;Q7</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>technology_integration;balance_multidimensional;spiritual_moral_anchor;contentment_acceptance;cultural_barrier</t>
+          <t>balance_multidimensional;policy_recommendation;practical_suggestion;spiritual_moral_anchor;training_deficit</t>
         </is>
       </c>
     </row>

</xml_diff>